<commit_message>
Add Playwright tests for login functionality and generate report
- Created a new test suite in `generated_test.py` for various login scenarios including valid and invalid credentials, empty fields, and special character handling.
- Added a `conftest.py` file to set up Playwright fixtures for browser interaction.
- Updated `test_login.py` to refactor the existing login test to use the new fixture and improved code structure.
- Introduced a new HTML report file `report.html` for test results.
- Updated the `testcases.xlsx` file to reflect the latest test cases.
</commit_message>
<xml_diff>
--- a/outputs/testcases.xlsx
+++ b/outputs/testcases.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,12 +441,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Successful login with valid credentials</t>
+          <t>Successful Login with Valid Credentials</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>User is successfully logged in and redirected to the dashboard or home page.</t>
+          <t>User is successfully logged in and redirected to the dashboard/home page.</t>
         </is>
       </c>
     </row>
@@ -458,12 +458,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Login with invalid username and valid password</t>
+          <t>Login with Invalid Username and Valid Password</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>An error message is displayed indicating invalid username or credentials. User remains on the login page.</t>
+          <t>An error message is displayed indicating 'Invalid username or password' (or similar).</t>
         </is>
       </c>
     </row>
@@ -475,12 +475,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Login with valid username and invalid password</t>
+          <t>Login with Valid Username and Invalid Password</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>An error message is displayed indicating invalid password or credentials. User remains on the login page.</t>
+          <t>An error message is displayed indicating 'Invalid username or password' (or similar).</t>
         </is>
       </c>
     </row>
@@ -492,12 +492,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Login with empty username and valid password</t>
+          <t>Login with Empty Username and Valid Password</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>An error message is displayed indicating that the username is required. User remains on the login page.</t>
+          <t>An error message is displayed indicating that the username is required.</t>
         </is>
       </c>
     </row>
@@ -509,12 +509,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Login with valid username and empty password</t>
+          <t>Login with Valid Username and Empty Password</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>An error message is displayed indicating that the password is required. User remains on the login page.</t>
+          <t>An error message is displayed indicating that the password is required.</t>
         </is>
       </c>
     </row>
@@ -526,12 +526,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Login with empty username and empty password</t>
+          <t>Login with Empty Username and Empty Password</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Error messages are displayed indicating that both username and password are required. User remains on the login page.</t>
+          <t>Error messages are displayed indicating that both username and password are required.</t>
         </is>
       </c>
     </row>
@@ -543,12 +543,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Login with special characters in username and valid password</t>
+          <t>Case Sensitivity of Username</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Depends on system's input validation. If special characters are allowed, user logs in. If not, an appropriate error message is shown.</t>
+          <t>The system should handle username case sensitivity according to its design. If case-insensitive, login should be successful. If case-sensitive, an error message should be displayed.</t>
         </is>
       </c>
     </row>
@@ -560,12 +560,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Login with special characters in password and valid username</t>
+          <t>Case Sensitivity of Password</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Depends on system's input validation. If special characters are allowed, user logs in. If not, an appropriate error message is shown.</t>
+          <t>An error message is displayed indicating 'Invalid username or password' (passwords are typically case-sensitive).</t>
         </is>
       </c>
     </row>
@@ -577,12 +577,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Case sensitivity of username</t>
+          <t>Attempt Login with Username containing Special Characters (if not allowed)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>User is successfully logged in and redirected to the dashboard or home page.</t>
+          <t>An error message is displayed indicating that the username contains invalid characters, or the login fails with an invalid credential message.</t>
         </is>
       </c>
     </row>
@@ -594,12 +594,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Case sensitivity of username (positive test)</t>
+          <t>Attempt Login with Password containing Special Characters (if allowed)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Depends on whether usernames are case-sensitive. If yes, user logs in. If no, user logs in if the system normalizes the input. If it requires exact match, and the stored username is lowercase, this might fail (leading to an error).</t>
+          <t>If the special characters are allowed in the password, the login should be successful. If not, an error message should be displayed.</t>
         </is>
       </c>
     </row>
@@ -611,12 +611,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Case sensitivity of password</t>
+          <t>Verify Password Masking</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>User is successfully logged in and redirected to the dashboard or home page.</t>
+          <t>The characters entered in the 'Password' field are masked (e.g., displayed as dots or asterisks).</t>
         </is>
       </c>
     </row>
@@ -628,12 +628,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Case sensitivity of password (positive test)</t>
+          <t>Login Button State - Enabled when fields are filled</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>User is successfully logged in and redirected to the dashboard or home page. Passwords are typically case-sensitive.</t>
+          <t>The 'Login' button is enabled.</t>
         </is>
       </c>
     </row>
@@ -645,63 +645,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Login with excessively long username</t>
+          <t>Login Button State - Disabled when fields are empty</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Depends on input validation. Either the input is truncated, an error message is displayed, or the login attempt might fail gracefully.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>TC_LOGIN_014</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Login with excessively long password</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Depends on input validation. Either the input is truncated, an error message is displayed, or the login attempt might fail gracefully.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>TC_LOGIN_015</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Login button disabled when fields are empty</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>The 'Login' button is disabled or visually indicates it's not clickable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>TC_LOGIN_016</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Login button enabled when fields are populated</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>The 'Login' button becomes enabled and clickable.</t>
+          <t>The 'Login' button is disabled by default.</t>
         </is>
       </c>
     </row>

</xml_diff>